<commit_message>
photo and txt works
</commit_message>
<xml_diff>
--- a/output/inStockInventory_20260916.xlsx
+++ b/output/inStockInventory_20260916.xlsx
@@ -130,7 +130,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2743200" cy="3876675"/>
@@ -153,9 +153,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2743200" cy="3876675"/>
@@ -178,9 +178,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>0</col>
+      <col>9</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2743200" cy="3876675"/>
@@ -203,12 +203,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>57</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2743200" cy="3876675"/>
+    <ext cx="2743200" cy="3867150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -216,31 +216,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>47</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2743200" cy="3867150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -543,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -619,432 +594,591 @@
     <row r="2">
       <c r="E2" t="inlineStr">
         <is>
-          <t>AS30188</t>
+          <t>FC19784</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BEIGE</t>
+          <t>BG</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>107</v>
+        <v>1000</v>
       </c>
       <c r="H2" t="n">
-        <v>23</v>
+        <v>12.25</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>AS60158 SET</t>
+          <t>80808</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>BG</t>
+          <t>LEO/BK</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="Q2" t="n">
-        <v>23.5</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="3">
       <c r="E3" t="inlineStr">
         <is>
-          <t>AS30188</t>
+          <t>FC19784</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BL</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>249</v>
+        <v>739</v>
       </c>
       <c r="H3" t="n">
-        <v>23</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>AS60158 SET</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>BK</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>357</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>23.5</v>
+        <v>12.25</v>
       </c>
     </row>
     <row r="4">
       <c r="E4" t="inlineStr">
         <is>
-          <t>AS30188</t>
+          <t>FC19784</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>BROWN</t>
+          <t>BLS</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>155</v>
+        <v>616</v>
       </c>
       <c r="H4" t="n">
-        <v>23</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>AS60158 SET</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>BR</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>174</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>23.5</v>
+        <v>12.25</v>
       </c>
     </row>
     <row r="5">
       <c r="E5" t="inlineStr">
         <is>
+          <t>FC19784</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FU</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" t="n">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>FC19784</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SAND</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1463</v>
+      </c>
+      <c r="H6" t="n">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>FC19784</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>TURQ</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>141</v>
+      </c>
+      <c r="H7" t="n">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>FC19784</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>21</v>
+      </c>
+      <c r="H8" t="n">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>163</v>
+      </c>
+      <c r="H12" t="n">
+        <v>23</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>AS60158</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>117</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>GY</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>89</v>
+      </c>
+      <c r="H13" t="n">
+        <v>23</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>AS60158</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>357</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>RBL</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>98</v>
+      </c>
+      <c r="H14" t="n">
+        <v>23</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>AS60158</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>174</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>RUST</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>62</v>
+      </c>
+      <c r="H15" t="n">
+        <v>23</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>AS60158</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>KHA</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>113</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>12</v>
+      </c>
+      <c r="H16" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" t="inlineStr">
+        <is>
           <t>AS30188</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>BEIGE</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>107</v>
+      </c>
+      <c r="H35" t="n">
+        <v>23</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>HL60121 SET</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>BGY</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>AS30188</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>BLACK</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>249</v>
+      </c>
+      <c r="H36" t="n">
+        <v>23</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>HL60121 SET</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>250</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>AS30188</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>BROWN</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>155</v>
+      </c>
+      <c r="H37" t="n">
+        <v>23</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>HL60121 SET</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>74</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>AS30188</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t>TAUPE</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="G38" t="n">
         <v>101</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H38" t="n">
         <v>23</v>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>AS60158 SET</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>HL60121 SET</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>105</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>HL60121 SET</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
         <is>
           <t>KHA</t>
         </is>
       </c>
-      <c r="P5" t="n">
-        <v>113</v>
-      </c>
-      <c r="Q5" t="n">
+      <c r="P39" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q39" t="n">
         <v>23.5</v>
       </c>
     </row>
-    <row r="25">
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>CR20202</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
+    <row r="40">
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>HL60121 SET</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>HL60143 SET</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>123</v>
+      </c>
+      <c r="H58" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>HOME - SHORTCUT</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>SKU HOME - SHORTCUT not found or search timed out</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>HL60143 SET</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
         <is>
           <t>BK</t>
         </is>
       </c>
-      <c r="G25" t="n">
-        <v>163</v>
-      </c>
-      <c r="H25" t="n">
-        <v>23</v>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>HL60121 SET</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>BGY</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>23.5</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>CR20202</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>GY</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>89</v>
-      </c>
-      <c r="H26" t="n">
-        <v>23</v>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>HL60121 SET</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>BK</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>250</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>23.5</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>CR20202</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>RBL</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>98</v>
-      </c>
-      <c r="H27" t="n">
-        <v>23</v>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>HL60121 SET</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="G59" t="n">
+        <v>434</v>
+      </c>
+      <c r="H59" t="n">
+        <v>23.25</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>HL60143 SET</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>BL</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>19</v>
+      </c>
+      <c r="H60" t="n">
+        <v>23.25</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>HL60143 SET</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
         <is>
           <t>BR</t>
         </is>
       </c>
-      <c r="P27" t="n">
-        <v>74</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>23.5</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>CR20202</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>RUST</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>62</v>
-      </c>
-      <c r="H28" t="n">
-        <v>23</v>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>HL60121 SET</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>105</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>23.5</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>CR20202</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="G61" t="n">
+        <v>202</v>
+      </c>
+      <c r="H61" t="n">
+        <v>23.25</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>HL60143 SET</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>KHA</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>101</v>
+      </c>
+      <c r="H62" t="n">
+        <v>23.25</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>HL60143 SET</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
         <is>
           <t>TP</t>
         </is>
       </c>
-      <c r="G29" t="n">
-        <v>12</v>
-      </c>
-      <c r="H29" t="n">
-        <v>23</v>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>HL60121 SET</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>KHA</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
-        <v>42</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>23.5</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>HL60121 SET</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="P30" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>23.5</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>HL60143 SET</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>BG</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>123</v>
-      </c>
-      <c r="H48" t="n">
-        <v>23.25</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>HL60143 SET</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>BK</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>434</v>
-      </c>
-      <c r="H49" t="n">
-        <v>23.25</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>HL60143 SET</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>BL</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>19</v>
-      </c>
-      <c r="H50" t="n">
-        <v>23.25</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>HL60143 SET</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>BR</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>202</v>
-      </c>
-      <c r="H51" t="n">
-        <v>23.25</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>HL60143 SET</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>KHA</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>101</v>
-      </c>
-      <c r="H52" t="n">
-        <v>23.25</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>HL60143 SET</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>TP</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
+      <c r="G63" t="n">
         <v>91</v>
       </c>
-      <c r="H53" t="n">
+      <c r="H63" t="n">
         <v>23.25</v>
       </c>
     </row>

</xml_diff>